<commit_message>
PF rule: REVISED_PF == ECR_PF (deposited); add side-by-side PF deducted/deposited/not-deposited columns
Per requirement, REVISED_PF now equals the ECR-filed (deposited) PF exactly,
every row (min-wage basic-floor uplift removed; 12% rule still holds since
B+D = ECR_PF/0.12). Added PF_WAGE_BASE_FULL, PF_DEDUCTED_12PCT,
PF_DEPOSITED_ECR, PF_NOT_DEPOSITED columns and rebuilt the consolidated
reconciliation summary across all 8 months.

https://claude.ai/code/session_015c3g1iE7rWC8fC3mEcXBS1
</commit_message>
<xml_diff>
--- a/PF_Reconciliation_Summary.xlsx
+++ b/PF_Reconciliation_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,32 +424,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Emp rows</t>
+          <t>PF deducted (12% B+D)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>PF members</t>
+          <t>PF deposited (ECR=REVISED)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ECR_PF filed</t>
+          <t>PF not deposited</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>REVISED_PF</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Diff (uplift)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Uplift rows</t>
+          <t>Rows short</t>
         </is>
       </c>
     </row>
@@ -460,22 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19161</v>
+        <v>25205249</v>
       </c>
       <c r="C2" t="n">
-        <v>16637</v>
+        <v>22929430</v>
       </c>
       <c r="D2" t="n">
-        <v>22929430</v>
+        <v>2275819</v>
       </c>
       <c r="E2" t="n">
-        <v>24392569</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1463139</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3037</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="3">
@@ -485,22 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19328</v>
+        <v>25179593</v>
       </c>
       <c r="C3" t="n">
-        <v>16648</v>
+        <v>22935027</v>
       </c>
       <c r="D3" t="n">
-        <v>22935027</v>
+        <v>2244566</v>
       </c>
       <c r="E3" t="n">
-        <v>24429395</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1494368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2913</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="4">
@@ -510,22 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18934</v>
+        <v>25146008</v>
       </c>
       <c r="C4" t="n">
-        <v>16778</v>
+        <v>23286410</v>
       </c>
       <c r="D4" t="n">
-        <v>23286410</v>
+        <v>1859598</v>
       </c>
       <c r="E4" t="n">
-        <v>24642976</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1356566</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2739</v>
+        <v>4480</v>
       </c>
     </row>
     <row r="5">
@@ -535,22 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19162</v>
+        <v>25974115</v>
       </c>
       <c r="C5" t="n">
-        <v>16934</v>
+        <v>23946516</v>
       </c>
       <c r="D5" t="n">
-        <v>23946516</v>
+        <v>2027599</v>
       </c>
       <c r="E5" t="n">
-        <v>25495410</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1548894</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2901</v>
+        <v>4757</v>
       </c>
     </row>
     <row r="6">
@@ -560,22 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19427</v>
+        <v>25406841</v>
       </c>
       <c r="C6" t="n">
-        <v>16782</v>
+        <v>23809892</v>
       </c>
       <c r="D6" t="n">
-        <v>23809892</v>
+        <v>1596949</v>
       </c>
       <c r="E6" t="n">
-        <v>25055940</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1246048</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2849</v>
+        <v>4541</v>
       </c>
     </row>
     <row r="7">
@@ -585,22 +545,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19205</v>
+        <v>25872554</v>
       </c>
       <c r="C7" t="n">
-        <v>17094</v>
+        <v>24354224</v>
       </c>
       <c r="D7" t="n">
-        <v>24354224</v>
+        <v>1518330</v>
       </c>
       <c r="E7" t="n">
-        <v>25620169</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1265945</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2760</v>
+        <v>4396</v>
       </c>
     </row>
     <row r="8">
@@ -610,22 +564,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19784</v>
+        <v>24131128</v>
       </c>
       <c r="C8" t="n">
-        <v>16853</v>
+        <v>24230628</v>
       </c>
       <c r="D8" t="n">
-        <v>24230628</v>
+        <v>-99500</v>
       </c>
       <c r="E8" t="n">
-        <v>24985552</v>
-      </c>
-      <c r="F8" t="n">
-        <v>754924</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2131</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="9">
@@ -635,22 +583,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19800</v>
+        <v>27124090</v>
       </c>
       <c r="C9" t="n">
-        <v>17439</v>
+        <v>25079121</v>
       </c>
       <c r="D9" t="n">
-        <v>25079121</v>
+        <v>2044969</v>
       </c>
       <c r="E9" t="n">
-        <v>26496046</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1416925</v>
-      </c>
-      <c r="G9" t="n">
-        <v>3055</v>
+        <v>4973</v>
       </c>
     </row>
     <row r="10">
@@ -660,22 +602,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>154801</v>
+        <v>204039578</v>
       </c>
       <c r="C10" t="n">
-        <v>135165</v>
+        <v>190571248</v>
       </c>
       <c r="D10" t="n">
-        <v>190571248</v>
+        <v>13468330</v>
       </c>
       <c r="E10" t="n">
-        <v>201118057</v>
-      </c>
-      <c r="F10" t="n">
-        <v>10546809</v>
-      </c>
-      <c r="G10" t="n">
-        <v>22385</v>
+        <v>36299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-detect header row (banner exports); add clean March; full 12-month PF reco
March was a raw export with a 3-line company banner above the header; the
reader now finds the EMPCODE header row automatically. All 12 months now
reconciled (REVISED_PF=ECR, all C1-C12 pass). Consolidated PF reconciliation
rebuilt across the full financial year.

https://claude.ai/code/session_015c3g1iE7rWC8fC3mEcXBS1
</commit_message>
<xml_diff>
--- a/PF_Reconciliation_Summary.xlsx
+++ b/PF_Reconciliation_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,22 +424,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Emp rows</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>PF deducted (12% B+D)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>PF deposited (ECR=REVISED)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>PF not deposited</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Rows short</t>
+          <t>PF not deposited (net)</t>
         </is>
       </c>
     </row>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>19161</v>
+      </c>
+      <c r="C2" t="n">
         <v>25205249</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>22929430</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2275819</v>
-      </c>
-      <c r="E2" t="n">
-        <v>5154</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>19327</v>
+      </c>
+      <c r="C3" t="n">
         <v>25179593</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>22935027</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>2244566</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4900</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>18933</v>
+      </c>
+      <c r="C4" t="n">
         <v>25146008</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>23286410</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>1859598</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4480</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>19162</v>
+      </c>
+      <c r="C5" t="n">
         <v>25974115</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>23946516</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2027599</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4757</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>19427</v>
+      </c>
+      <c r="C6" t="n">
         <v>25406841</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>23809892</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1596949</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4541</v>
       </c>
     </row>
     <row r="7">
@@ -545,16 +545,16 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>19205</v>
+      </c>
+      <c r="C7" t="n">
         <v>25872554</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>24354224</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>1518330</v>
-      </c>
-      <c r="E7" t="n">
-        <v>4396</v>
       </c>
     </row>
     <row r="8">
@@ -564,54 +564,130 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>19784</v>
+      </c>
+      <c r="C8" t="n">
         <v>24131128</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>24230628</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>-99500</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3098</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>December</t>
+          <t>November</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27124090</v>
+        <v>19296</v>
       </c>
       <c r="C9" t="n">
-        <v>25079121</v>
+        <v>25419195</v>
       </c>
       <c r="D9" t="n">
-        <v>2044969</v>
+        <v>23801945</v>
       </c>
       <c r="E9" t="n">
-        <v>4973</v>
+        <v>1617250</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>December</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>204039578</v>
+        <v>19799</v>
       </c>
       <c r="C10" t="n">
-        <v>190571248</v>
+        <v>27124090</v>
       </c>
       <c r="D10" t="n">
-        <v>13468330</v>
+        <v>25079121</v>
       </c>
       <c r="E10" t="n">
-        <v>36299</v>
+        <v>2044969</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20364</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27438064</v>
+      </c>
+      <c r="D11" t="n">
+        <v>25587803</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1850261</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>19862</v>
+      </c>
+      <c r="C12" t="n">
+        <v>27217117</v>
+      </c>
+      <c r="D12" t="n">
+        <v>25462898</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1754219</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20749</v>
+      </c>
+      <c r="C13" t="n">
+        <v>27729272</v>
+      </c>
+      <c r="D13" t="n">
+        <v>25757367</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1971905</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TOTAL (FY)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>235069</v>
+      </c>
+      <c r="C14" t="n">
+        <v>311843226</v>
+      </c>
+      <c r="D14" t="n">
+        <v>291181261</v>
+      </c>
+      <c r="E14" t="n">
+        <v>20661965</v>
       </c>
     </row>
   </sheetData>

</xml_diff>